<commit_message>
Migrate urop/prospective-students; repackage JCR (9 pages)
- Add source HTML for /urop/prospective-students at proper subtree path.
  Reuses the department-landing template (no code change): interior shell dropped
  as chrome, #page-content is pure default content — a YouTube video (iframe
  converted to a link per EDS video convention; cleanup drops raw iframes), an
  intro paragraph, and a stack of 7 full-width CTA buttons (each a program link).
  No block instances (four-button selector simply doesn't match here).
- page-templates.json: add urop URL + broaden department-landing description.
- generate-jcr.mjs: add /urop/prospective-students → content/lsa-eds-ue/urop/prospective-students.
- Rebuild dist/lsa-eds-ue-content.zip → now 9/9 pages, all well-formed XML.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-department-landing.report.xlsx
+++ b/tools/importer/reports/import-department-landing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="82">
   <si>
     <t>_reportFile</t>
   </si>
@@ -199,6 +199,24 @@
     <t>http://localhost:8082/lsa/prospective-students.html</t>
   </si>
   <si>
+    <t>urop/prospective-students.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>urop/prospective-students</t>
+  </si>
+  <si>
+    <t>2026-08-14T15:54:22.361Z</t>
+  </si>
+  <si>
+    <t>Prospective UROP Students | U-M LSA UROP: A Center for Research, Scholarship, and Creative Inquiry</t>
+  </si>
+  <si>
+    <t>http://localhost:8082/urop/prospective-students.html</t>
+  </si>
+  <si>
     <t>lsa/academics/departments-and-units.html.report.json</t>
   </si>
   <si>
@@ -225,9 +243,6 @@
   </si>
   <si>
     <t>lsa/academics/departments-and-units.report.json</t>
-  </si>
-  <si>
-    <t>[]</t>
   </si>
   <si>
     <t>lsa/academics/departments-and-units</t>
@@ -643,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
@@ -974,31 +989,31 @@
         <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
         <v>62</v>
       </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" t="s">
+        <v>49</v>
+      </c>
+      <c r="I10" t="s">
         <v>63</v>
       </c>
-      <c r="G10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>64</v>
-      </c>
-      <c r="J10" t="s">
-        <v>12</v>
       </c>
       <c r="K10" t="s">
         <v>65</v>
@@ -1009,34 +1024,34 @@
         <v>66</v>
       </c>
       <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
         <v>67</v>
       </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="E11" t="s">
         <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="I11" t="s">
         <v>70</v>
       </c>
       <c r="J11" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11" t="s">
         <v>71</v>
-      </c>
-      <c r="K11" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1044,7 +1059,7 @@
         <v>72</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
@@ -1062,16 +1077,51 @@
         <v>22</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="I12" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" t="s">
+        <v>76</v>
+      </c>
+      <c r="K12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" t="s">
         <v>74</v>
       </c>
-      <c r="J12" t="s">
-        <v>75</v>
-      </c>
-      <c r="K12" t="s">
-        <v>76</v>
+      <c r="I13" t="s">
+        <v>79</v>
+      </c>
+      <c r="J13" t="s">
+        <v>80</v>
+      </c>
+      <c r="K13" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>